<commit_message>
Organization and more paper writing
</commit_message>
<xml_diff>
--- a/analysis/2025-10-30 Tables for Report.xlsx
+++ b/analysis/2025-10-30 Tables for Report.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Personal\Coach_WAR\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91EB18AE-11C4-4A89-93ED-F13A9157D3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5990A4C-CFA1-40C9-944A-C2F70303F538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="6" xr2:uid="{E7B8E32F-0AEC-4226-BFE4-04A50A9DFAB8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="9" xr2:uid="{E7B8E32F-0AEC-4226-BFE4-04A50A9DFAB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Features by Cat" sheetId="2" r:id="rId1"/>
@@ -20,6 +20,9 @@
     <sheet name="Top Seasons" sheetId="5" r:id="rId5"/>
     <sheet name="Top Averages" sheetId="6" r:id="rId6"/>
     <sheet name="By Decade" sheetId="7" r:id="rId7"/>
+    <sheet name="Off vs Def" sheetId="8" r:id="rId8"/>
+    <sheet name="Validation" sheetId="9" r:id="rId9"/>
+    <sheet name="Persistence" sheetId="10" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Top Averages'!$H$20:$M$20</definedName>
@@ -67,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1309" uniqueCount="858">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="965">
   <si>
     <t>Win_Pct</t>
   </si>
@@ -2640,7 +2643,334 @@
     <t>Delta, 2020's vs. 1970s</t>
   </si>
   <si>
-    <t>Avg. Coach WAR per Season</t>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Test Type                       </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Test Statistic </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> p-value </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Effect Size        </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Interpretation             </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>---------------------------------</t>
+  </si>
+  <si>
+    <t>----------------</t>
+  </si>
+  <si>
+    <t>--------------------</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Welch's t-test (parametric)     </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> t = -1.642     </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cohen's d = -0.086 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Not significant            </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mann-Whitney U (non-parametric) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> U = 260,162    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -                  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Background </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Coaches </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Seasons </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mean WAR </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Median WAR </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Std Dev </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Offensive  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Defensive  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Difference </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -       </t>
+  </si>
+  <si>
+    <t>Difference</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Marginally significant</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mann-Whitney U test Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Decade </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sample Sizes (O/D)           </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mean WAR (O/D)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Mann-Whitney U   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Cohen's d </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Significance </t>
+  </si>
+  <si>
+    <t>--------</t>
+  </si>
+  <si>
+    <t>------------------------------</t>
+  </si>
+  <si>
+    <t>------------------</t>
+  </si>
+  <si>
+    <t>-----------</t>
+  </si>
+  <si>
+    <t>--------------</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Coaches / Seasons            </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> games/season    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> O - D      </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> U-stat / p-value </t>
+  </si>
+  <si>
+    <t xml:space="preserve">           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1970s  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -0.355 / +0.573 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3290p = 0.0001   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> **           </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1980s  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> +0.421 / +0.456 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 5389p = 0.555    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -            </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1990s  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> -0.140 / +0.193 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 7553p = 0.211    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2000s  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> +0.139 / +0.076 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 10275p = 0.763   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2010s  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> +0.246 / +0.528 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 9430p = 0.234    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 2020s  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> +0.572 / +0.156 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3151p = 0.159    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 38/24 coaches, 95/101 seasons  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 32/19 coaches, 149/76 seasons  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 38/25 coaches, 163/102 seasons </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 42/33 coaches, 165/122 seasons </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 44/32 coaches, 163/126 seasons </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 33/22 coaches, 91/61 seasons   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Difference (O - D)</t>
+  </si>
+  <si>
+    <t>U-statistic</t>
+  </si>
+  <si>
+    <t>p-value</t>
+  </si>
+  <si>
+    <t>Highly Significant</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Sample Size, Coaches (O/D)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Validation Strategy          </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Training Samples                           </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Test Samples                          </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Train R² </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Test R² </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Test RMSE </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Generalization Gap </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Temporal Holdout (2020-2024) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Holdout Coaches              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> New Coaches in Modern Era    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1,523 seasons 
+(1970-2019)                   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1,363 seasons
+(216 coaches)                 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1,652 seasons
+(pre-2020 + 80% of 2020-2024) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 160 seasons
+(2020-2024)                </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 320 seasons
+(54 coaches)               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 31 seasons
+(11 new coaches, 2020-2024) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Quintile    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Year N WAR (games) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Year N+1 WAR (games) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Change (games) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> % Retained </t>
+  </si>
+  <si>
+    <t>----------------------</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Q1 (Worst)  </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Q2          </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Q3 (Middle) </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> N/A        </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Q4          </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Q5 (Best)   </t>
   </si>
 </sst>
 </file>
@@ -2649,7 +2979,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -2686,15 +3016,21 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -2892,13 +3228,137 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top style="double">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
         <color indexed="64"/>
       </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -2909,8 +3369,10 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="double">
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -2920,8 +3382,10 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom style="double">
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -2936,33 +3400,7 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="double">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -2971,7 +3409,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3098,13 +3536,13 @@
     <xf numFmtId="2" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3122,32 +3560,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3158,23 +3584,170 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3663,6 +4236,268 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAD42C9B-D870-448B-8B15-7E5FEE5BEFC2}">
+  <dimension ref="B1:G15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="20"/>
+    <col min="2" max="6" width="17.08984375" style="20" customWidth="1"/>
+    <col min="7" max="8" width="14.90625" style="20" customWidth="1"/>
+    <col min="9" max="16384" width="8.7265625" style="20"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:7" s="55" customFormat="1" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="51" t="str" cm="1">
+        <f t="array" ref="B2:F2">TRIM(C9:G9)</f>
+        <v>Quintile</v>
+      </c>
+      <c r="C2" s="52" t="str">
+        <v>Year N WAR (games)</v>
+      </c>
+      <c r="D2" s="52" t="str">
+        <v>Year N+1 WAR (games)</v>
+      </c>
+      <c r="E2" s="52" t="str">
+        <v>Change (games)</v>
+      </c>
+      <c r="F2" s="54" t="str">
+        <v>% Retained</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="108" t="str" cm="1">
+        <f t="array" ref="B3:B7">C11:C15</f>
+        <v xml:space="preserve"> Q1 (Worst)  </v>
+      </c>
+      <c r="C3" s="112" cm="1">
+        <f t="array" ref="C3:F7">IFERROR(VALUE(D11:G15),TRIM(D11:G15))</f>
+        <v>-2.33</v>
+      </c>
+      <c r="D3" s="112">
+        <v>-0.93</v>
+      </c>
+      <c r="E3" s="64">
+        <v>1.4</v>
+      </c>
+      <c r="F3" s="45">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B4" s="111" t="str">
+        <v xml:space="preserve"> Q2          </v>
+      </c>
+      <c r="C4" s="113">
+        <v>-0.77</v>
+      </c>
+      <c r="D4" s="113">
+        <v>-0.59</v>
+      </c>
+      <c r="E4" s="114">
+        <v>0.18</v>
+      </c>
+      <c r="F4" s="65">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B5" s="111" t="str">
+        <v xml:space="preserve"> Q3 (Middle) </v>
+      </c>
+      <c r="C5" s="113">
+        <v>0.17</v>
+      </c>
+      <c r="D5" s="113">
+        <v>-0.1</v>
+      </c>
+      <c r="E5" s="114">
+        <v>-0.27</v>
+      </c>
+      <c r="F5" s="65" t="str">
+        <v>N/A</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B6" s="109" t="str">
+        <v xml:space="preserve"> Q4          </v>
+      </c>
+      <c r="C6" s="115">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="D6" s="115">
+        <v>0.35</v>
+      </c>
+      <c r="E6" s="116">
+        <v>-0.8</v>
+      </c>
+      <c r="F6" s="46">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="110" t="str">
+        <v xml:space="preserve"> Q5 (Best)   </v>
+      </c>
+      <c r="C7" s="117">
+        <v>2.64</v>
+      </c>
+      <c r="D7" s="117">
+        <v>0.65</v>
+      </c>
+      <c r="E7" s="118">
+        <v>-1.99</v>
+      </c>
+      <c r="F7" s="47">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B9" s="20" t="s">
+        <v>857</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>953</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>954</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>955</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>956</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B10" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>776</v>
+      </c>
+      <c r="D10" s="55" t="s">
+        <v>866</v>
+      </c>
+      <c r="E10" s="55" t="s">
+        <v>958</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>865</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B11" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>959</v>
+      </c>
+      <c r="D11" s="119">
+        <v>-2.33</v>
+      </c>
+      <c r="E11" s="119">
+        <v>-0.93</v>
+      </c>
+      <c r="F11" s="120">
+        <v>1.4</v>
+      </c>
+      <c r="G11" s="120">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>960</v>
+      </c>
+      <c r="D12" s="119">
+        <v>-0.77</v>
+      </c>
+      <c r="E12" s="119">
+        <v>-0.59</v>
+      </c>
+      <c r="F12" s="120">
+        <v>0.18</v>
+      </c>
+      <c r="G12" s="120">
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B13" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>961</v>
+      </c>
+      <c r="D13" s="120">
+        <v>0.17</v>
+      </c>
+      <c r="E13" s="120">
+        <v>-0.1</v>
+      </c>
+      <c r="F13" s="120">
+        <v>-0.27</v>
+      </c>
+      <c r="G13" s="120" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B14" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>963</v>
+      </c>
+      <c r="D14" s="120">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="E14" s="120">
+        <v>0.35</v>
+      </c>
+      <c r="F14" s="120">
+        <v>-0.8</v>
+      </c>
+      <c r="G14" s="120">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B15" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>964</v>
+      </c>
+      <c r="D15" s="120">
+        <v>2.64</v>
+      </c>
+      <c r="E15" s="120">
+        <v>0.65</v>
+      </c>
+      <c r="F15" s="120">
+        <v>-1.99</v>
+      </c>
+      <c r="G15" s="120">
+        <v>0.25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{129F9831-1725-4379-93CD-2DC6DD2D8C52}">
   <sheetPr codeName="Sheet2"/>
@@ -11778,235 +12613,1242 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A52C07A-37FD-4FD9-80F8-E4D4E39D4100}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="B1:I13"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="B2:K32"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="20"/>
-    <col min="2" max="2" width="12.08984375" style="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.54296875" style="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" style="57" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" style="40" customWidth="1"/>
+    <col min="5" max="7" width="14.54296875" style="20" customWidth="1"/>
+    <col min="8" max="8" width="14.54296875" style="40" customWidth="1"/>
+    <col min="9" max="9" width="13.6328125" style="40" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="16384" width="8.7265625" style="20"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="88"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2" s="89"/>
+    </row>
+    <row r="3" spans="2:9" s="55" customFormat="1" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="61" t="s">
+        <v>845</v>
+      </c>
+      <c r="C3" s="23" t="str" cm="1">
+        <f t="array" ref="C3:H3">_xlfn.SEQUENCE(1,6,1970,10)&amp;"'s"</f>
+        <v>1970's</v>
+      </c>
+      <c r="D3" s="23" t="str">
+        <v>1980's</v>
+      </c>
+      <c r="E3" s="23" t="str">
+        <v>1990's</v>
+      </c>
+      <c r="F3" s="23" t="str">
+        <v>2000's</v>
+      </c>
+      <c r="G3" s="23" t="str">
+        <v>2010's</v>
+      </c>
+      <c r="H3" s="24" t="str">
+        <v>2020's</v>
+      </c>
+      <c r="I3" s="54" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="28" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="62" t="s">
+        <v>848</v>
+      </c>
+      <c r="C4" s="64" cm="1">
+        <f t="array" ref="C4:H4">C19:H19</f>
+        <v>-0.35</v>
+      </c>
+      <c r="D4" s="64">
+        <v>0.42</v>
+      </c>
+      <c r="E4" s="64">
+        <v>-0.14000000000000001</v>
+      </c>
+      <c r="F4" s="64">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="G4" s="64">
+        <v>0.25</v>
+      </c>
+      <c r="H4" s="45">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="I4" s="65">
+        <f t="shared" ref="I4:I6" si="0">H4-C4</f>
+        <v>0.91999999999999993</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="71" t="s">
+        <v>847</v>
+      </c>
+      <c r="C5" s="103" cm="1">
+        <f t="array" ref="C5:H5">C18:H18</f>
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="D5" s="103">
+        <v>0.46</v>
+      </c>
+      <c r="E5" s="103">
+        <v>0.19</v>
+      </c>
+      <c r="F5" s="103">
+        <v>0.08</v>
+      </c>
+      <c r="G5" s="103">
+        <v>0.53</v>
+      </c>
+      <c r="H5" s="104">
+        <v>0.16</v>
+      </c>
+      <c r="I5" s="46">
+        <f t="shared" si="0"/>
+        <v>-0.40999999999999992</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" ht="28" hidden="1" customHeight="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B6" s="100" t="s">
+        <v>849</v>
+      </c>
+      <c r="C6" s="101"/>
+      <c r="D6" s="101"/>
+      <c r="E6" s="101"/>
+      <c r="F6" s="101"/>
+      <c r="G6" s="101"/>
+      <c r="H6" s="102"/>
+      <c r="I6" s="47">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" s="55" customFormat="1" ht="28" customHeight="1" collapsed="1" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="94" t="s">
+        <v>936</v>
+      </c>
+      <c r="C7" s="90" t="str" cm="1">
+        <f t="array" ref="C7:H7">TRIM(_xlfn.TEXTBEFORE(TRANSPOSE(C27:C32),"coaches"))</f>
+        <v>38/24</v>
+      </c>
+      <c r="D7" s="90" t="str">
+        <v>32/19</v>
+      </c>
+      <c r="E7" s="90" t="str">
+        <v>38/25</v>
+      </c>
+      <c r="F7" s="90" t="str">
+        <v>42/33</v>
+      </c>
+      <c r="G7" s="90" t="str">
+        <v>44/32</v>
+      </c>
+      <c r="H7" s="95" t="str">
+        <v>33/22</v>
+      </c>
+      <c r="I7" s="91"/>
+    </row>
+    <row r="8" spans="2:9" s="55" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="96" t="str">
+        <f>SUBSTITUTE(B7,"Coaches", "Seasons")</f>
+        <v>Sample Size, Seasons (O/D)</v>
+      </c>
+      <c r="C8" s="97" t="str" cm="1">
+        <f t="array" ref="C8:H8">TRIM(_xlfn.TEXTBEFORE(_xlfn.TEXTAFTER(TRANSPOSE(C27:C32),","),"seasons"))</f>
+        <v>95/101</v>
+      </c>
+      <c r="D8" s="97" t="str">
+        <v>149/76</v>
+      </c>
+      <c r="E8" s="97" t="str">
+        <v>163/102</v>
+      </c>
+      <c r="F8" s="97" t="str">
+        <v>165/122</v>
+      </c>
+      <c r="G8" s="97" t="str">
+        <v>163/126</v>
+      </c>
+      <c r="H8" s="98" t="str">
+        <v>91/61</v>
+      </c>
+      <c r="I8" s="99"/>
+    </row>
+    <row r="9" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="78" t="str" cm="1">
+        <f t="array" ref="B9:B10">TRIM(TRANSPOSE(D24:E24))</f>
+        <v>Mean WAR (O/D)</v>
+      </c>
+      <c r="C9" s="32" t="str" cm="1">
+        <f t="array" ref="C9:H10">TRIM(TRANSPOSE(D27:E32))</f>
+        <v>-0.355 / +0.573</v>
+      </c>
+      <c r="D9" s="32" t="str">
+        <v>+0.421 / +0.456</v>
+      </c>
+      <c r="E9" s="32" t="str">
+        <v>-0.140 / +0.193</v>
+      </c>
+      <c r="F9" s="32" t="str">
+        <v>+0.139 / +0.076</v>
+      </c>
+      <c r="G9" s="32" t="str">
+        <v>+0.246 / +0.528</v>
+      </c>
+      <c r="H9" s="34" t="str">
+        <v>+0.572 / +0.156</v>
+      </c>
+      <c r="I9" s="92"/>
+    </row>
+    <row r="10" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="78" t="str">
+        <v>Difference (O - D)</v>
+      </c>
+      <c r="C10" s="32" t="str">
+        <v>-0.927</v>
+      </c>
+      <c r="D10" s="32" t="str">
+        <v>-0.035</v>
+      </c>
+      <c r="E10" s="32" t="str">
+        <v>-0.333</v>
+      </c>
+      <c r="F10" s="32" t="str">
+        <v>0.063</v>
+      </c>
+      <c r="G10" s="32" t="str">
+        <v>-0.282</v>
+      </c>
+      <c r="H10" s="34" t="str">
+        <v>0.416</v>
+      </c>
+      <c r="I10" s="92"/>
+    </row>
+    <row r="11" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="78" t="str" cm="1">
+        <f t="array" ref="B11:B12">TRANSPOSE(J24:K24)</f>
+        <v>U-statistic</v>
+      </c>
+      <c r="C11" s="32" cm="1">
+        <f t="array" ref="C11:H12">TRANSPOSE(J27:K32)</f>
+        <v>3290</v>
+      </c>
+      <c r="D11" s="32">
+        <v>5389</v>
+      </c>
+      <c r="E11" s="32">
+        <v>7553</v>
+      </c>
+      <c r="F11" s="32">
+        <v>10275</v>
+      </c>
+      <c r="G11" s="32">
+        <v>9430</v>
+      </c>
+      <c r="H11" s="34">
+        <v>3151</v>
+      </c>
+      <c r="I11" s="92"/>
+    </row>
+    <row r="12" spans="2:9" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="78" t="str">
+        <v>p-value</v>
+      </c>
+      <c r="C12" s="32">
+        <v>1E-4</v>
+      </c>
+      <c r="D12" s="32">
+        <v>0.55500000000000005</v>
+      </c>
+      <c r="E12" s="32">
+        <v>0.21099999999999999</v>
+      </c>
+      <c r="F12" s="32">
+        <v>0.76300000000000001</v>
+      </c>
+      <c r="G12" s="32">
+        <v>0.23400000000000001</v>
+      </c>
+      <c r="H12" s="34">
+        <v>0.159</v>
+      </c>
+      <c r="I12" s="92"/>
+    </row>
+    <row r="13" spans="2:9" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B13" s="83" t="str">
+        <f>TRIM(H24)</f>
+        <v>Significance</v>
+      </c>
+      <c r="C13" s="37" t="s">
+        <v>934</v>
+      </c>
+      <c r="D13" s="37" t="s">
+        <v>935</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>935</v>
+      </c>
+      <c r="F13" s="37" t="s">
+        <v>935</v>
+      </c>
+      <c r="G13" s="37" t="s">
+        <v>935</v>
+      </c>
+      <c r="H13" s="39" t="s">
+        <v>935</v>
+      </c>
+      <c r="I13" s="93"/>
+    </row>
+    <row r="16" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B16" s="20" t="s">
+        <v>846</v>
+      </c>
+      <c r="C16" s="57" t="s">
+        <v>850</v>
+      </c>
+      <c r="D16" s="40" t="s">
+        <v>851</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>852</v>
+      </c>
+      <c r="F16" s="20" t="s">
+        <v>853</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>854</v>
+      </c>
+      <c r="H16" s="40" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="17" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B17" s="20" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="18" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B18" s="20" t="s">
+        <v>847</v>
+      </c>
+      <c r="C18" s="57">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="D18" s="40">
+        <v>0.46</v>
+      </c>
+      <c r="E18" s="20">
+        <v>0.19</v>
+      </c>
+      <c r="F18" s="20">
+        <v>0.08</v>
+      </c>
+      <c r="G18" s="20">
+        <v>0.53</v>
+      </c>
+      <c r="H18" s="40">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B19" s="20" t="s">
+        <v>848</v>
+      </c>
+      <c r="C19" s="57">
+        <v>-0.35</v>
+      </c>
+      <c r="D19" s="40">
+        <v>0.42</v>
+      </c>
+      <c r="E19" s="20">
+        <v>-0.14000000000000001</v>
+      </c>
+      <c r="F19" s="20">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="G19" s="20">
+        <v>0.25</v>
+      </c>
+      <c r="H19" s="40">
+        <v>0.56999999999999995</v>
+      </c>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B20" s="20" t="s">
+        <v>849</v>
+      </c>
+      <c r="C20" s="57">
+        <v>0.02</v>
+      </c>
+      <c r="D20" s="40">
+        <v>-0.11</v>
+      </c>
+      <c r="E20" s="20">
+        <v>0.51</v>
+      </c>
+      <c r="F20" s="20">
+        <v>0.04</v>
+      </c>
+      <c r="G20" s="20">
+        <v>0.43</v>
+      </c>
+      <c r="H20" s="40">
+        <v>-7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="2:11" s="55" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+      <c r="B24" s="67" t="s">
+        <v>887</v>
+      </c>
+      <c r="C24" s="68" t="s">
+        <v>888</v>
+      </c>
+      <c r="D24" s="55" t="s">
+        <v>889</v>
+      </c>
+      <c r="E24" s="55" t="s">
+        <v>931</v>
+      </c>
+      <c r="F24" s="55" t="s">
+        <v>890</v>
+      </c>
+      <c r="G24" s="68" t="s">
+        <v>891</v>
+      </c>
+      <c r="H24" s="68" t="s">
+        <v>892</v>
+      </c>
+      <c r="I24" s="68"/>
+      <c r="J24" s="55" t="s">
+        <v>932</v>
+      </c>
+      <c r="K24" s="55" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B25" s="57" t="s">
+        <v>893</v>
+      </c>
+      <c r="C25" s="40" t="s">
+        <v>894</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>778</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>795</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>895</v>
+      </c>
+      <c r="G25" s="40" t="s">
+        <v>896</v>
+      </c>
+      <c r="H25" s="40" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B26" s="57" t="s">
+        <v>898</v>
+      </c>
+      <c r="C26" s="40" t="s">
+        <v>899</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>900</v>
+      </c>
+      <c r="E26" s="20" t="s">
+        <v>901</v>
+      </c>
+      <c r="F26" s="20" t="s">
+        <v>902</v>
+      </c>
+      <c r="G26" s="40" t="s">
+        <v>903</v>
+      </c>
+      <c r="H26" s="40" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="27" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B27" s="57" t="s">
+        <v>905</v>
+      </c>
+      <c r="C27" s="40" t="s">
+        <v>925</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>906</v>
+      </c>
+      <c r="E27" s="20">
+        <v>-0.92700000000000005</v>
+      </c>
+      <c r="F27" s="20" t="s">
+        <v>907</v>
+      </c>
+      <c r="G27" s="40">
+        <v>-0.53200000000000003</v>
+      </c>
+      <c r="H27" s="40" t="s">
+        <v>908</v>
+      </c>
+      <c r="J27" s="20" cm="1">
+        <f t="array" ref="J27:J32">VALUE(_xlfn.TEXTBEFORE(F27:F32,"p"))</f>
+        <v>3290</v>
+      </c>
+      <c r="K27" s="20" cm="1">
+        <f t="array" ref="K27:K32">VALUE(_xlfn.TEXTAFTER(F27:F32,"="))</f>
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B28" s="57" t="s">
+        <v>909</v>
+      </c>
+      <c r="C28" s="40" t="s">
+        <v>926</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>910</v>
+      </c>
+      <c r="E28" s="20">
+        <v>-3.5000000000000003E-2</v>
+      </c>
+      <c r="F28" s="20" t="s">
+        <v>911</v>
+      </c>
+      <c r="G28" s="40">
+        <v>-1.9E-2</v>
+      </c>
+      <c r="H28" s="40" t="s">
+        <v>912</v>
+      </c>
+      <c r="J28" s="20">
+        <v>5389</v>
+      </c>
+      <c r="K28" s="20">
+        <v>0.55500000000000005</v>
+      </c>
+    </row>
+    <row r="29" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B29" s="57" t="s">
+        <v>913</v>
+      </c>
+      <c r="C29" s="40" t="s">
+        <v>927</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>914</v>
+      </c>
+      <c r="E29" s="20">
+        <v>-0.33300000000000002</v>
+      </c>
+      <c r="F29" s="20" t="s">
+        <v>915</v>
+      </c>
+      <c r="G29" s="40">
+        <v>-0.17399999999999999</v>
+      </c>
+      <c r="H29" s="40" t="s">
+        <v>912</v>
+      </c>
+      <c r="J29" s="20">
+        <v>7553</v>
+      </c>
+      <c r="K29" s="20">
+        <v>0.21099999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B30" s="57" t="s">
+        <v>916</v>
+      </c>
+      <c r="C30" s="40" t="s">
+        <v>928</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>917</v>
+      </c>
+      <c r="E30" s="20">
+        <v>6.3E-2</v>
+      </c>
+      <c r="F30" s="20" t="s">
+        <v>918</v>
+      </c>
+      <c r="G30" s="40">
+        <v>3.5000000000000003E-2</v>
+      </c>
+      <c r="H30" s="40" t="s">
+        <v>912</v>
+      </c>
+      <c r="J30" s="20">
+        <v>10275</v>
+      </c>
+      <c r="K30" s="20">
+        <v>0.76300000000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B31" s="57" t="s">
+        <v>919</v>
+      </c>
+      <c r="C31" s="40" t="s">
+        <v>929</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>920</v>
+      </c>
+      <c r="E31" s="20">
+        <v>-0.28199999999999997</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>921</v>
+      </c>
+      <c r="G31" s="40">
+        <v>-0.151</v>
+      </c>
+      <c r="H31" s="40" t="s">
+        <v>912</v>
+      </c>
+      <c r="J31" s="20">
+        <v>9430</v>
+      </c>
+      <c r="K31" s="20">
+        <v>0.23400000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="2:11" x14ac:dyDescent="0.35">
+      <c r="B32" s="57" t="s">
+        <v>922</v>
+      </c>
+      <c r="C32" s="40" t="s">
+        <v>930</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>923</v>
+      </c>
+      <c r="E32" s="20">
+        <v>0.41599999999999998</v>
+      </c>
+      <c r="F32" s="20" t="s">
+        <v>924</v>
+      </c>
+      <c r="G32" s="40">
+        <v>0.25700000000000001</v>
+      </c>
+      <c r="H32" s="40" t="s">
+        <v>912</v>
+      </c>
+      <c r="J32" s="20">
+        <v>3151</v>
+      </c>
+      <c r="K32" s="20">
+        <v>0.159</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3A2CB53-2941-4642-9382-91358B7FAA54}">
+  <dimension ref="B2:I26"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="20"/>
+    <col min="2" max="2" width="13" style="20" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.08984375" style="57" customWidth="1"/>
     <col min="4" max="4" width="9.08984375" style="40" customWidth="1"/>
     <col min="5" max="7" width="9.08984375" style="20" customWidth="1"/>
-    <col min="8" max="8" width="9.08984375" style="40" customWidth="1"/>
+    <col min="8" max="8" width="19.453125" style="40" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.6328125" style="40" customWidth="1"/>
     <col min="10" max="16384" width="8.7265625" style="20"/>
   </cols>
   <sheetData>
+    <row r="2" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+      <c r="F2"/>
+      <c r="G2"/>
+      <c r="H2"/>
+      <c r="I2"/>
+    </row>
+    <row r="3" spans="2:9" s="55" customFormat="1" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="66" t="s">
+        <v>845</v>
+      </c>
+      <c r="C3" s="52" t="str" cm="1">
+        <f t="array" ref="C3:G3">D16:H16</f>
+        <v xml:space="preserve"> Coaches </v>
+      </c>
+      <c r="D3" s="52" t="str">
+        <v xml:space="preserve"> Seasons </v>
+      </c>
+      <c r="E3" s="52" t="str">
+        <v xml:space="preserve"> Mean WAR </v>
+      </c>
+      <c r="F3" s="52" t="str">
+        <v xml:space="preserve"> Median WAR </v>
+      </c>
+      <c r="G3" s="72" t="str">
+        <v xml:space="preserve"> Std Dev </v>
+      </c>
+      <c r="H3" s="75" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="62" t="s">
+        <v>847</v>
+      </c>
+      <c r="C4" s="69" cm="1">
+        <f t="array" ref="C4:G4">D19:H19</f>
+        <v>112</v>
+      </c>
+      <c r="D4" s="69">
+        <v>639</v>
+      </c>
+      <c r="E4" s="28">
+        <v>1.52E-2</v>
+      </c>
+      <c r="F4" s="28">
+        <v>1.8499999999999999E-2</v>
+      </c>
+      <c r="G4" s="73">
+        <v>0.1111</v>
+      </c>
+      <c r="H4" s="76"/>
+      <c r="I4" s="20"/>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B5" s="63" t="s">
+        <v>848</v>
+      </c>
+      <c r="C5" s="70" cm="1">
+        <f t="array" ref="C5:G5">D18:H18</f>
+        <v>154</v>
+      </c>
+      <c r="D5" s="70">
+        <v>860</v>
+      </c>
+      <c r="E5" s="33">
+        <v>5.4999999999999997E-3</v>
+      </c>
+      <c r="F5" s="33">
+        <v>2.3E-3</v>
+      </c>
+      <c r="G5" s="74">
+        <v>0.1134</v>
+      </c>
+      <c r="H5" s="77"/>
+      <c r="I5" s="20"/>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+      <c r="B6" s="63" t="s">
+        <v>884</v>
+      </c>
+      <c r="C6" s="70" cm="1">
+        <f t="array" ref="C6:G6">_xlfn.ANCHORARRAY(C5)-_xlfn.ANCHORARRAY(C4)</f>
+        <v>42</v>
+      </c>
+      <c r="D6" s="70">
+        <v>221</v>
+      </c>
+      <c r="E6" s="33">
+        <v>-9.7000000000000003E-3</v>
+      </c>
+      <c r="F6" s="33">
+        <v>-1.6199999999999999E-2</v>
+      </c>
+      <c r="G6" s="74">
+        <v>2.2999999999999965E-3</v>
+      </c>
+      <c r="H6" s="77"/>
+      <c r="I6" s="20"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B7" s="78" t="str" cm="1">
+        <f t="array" ref="B7:B10">TRIM(TRANSPOSE(D23:G23))</f>
+        <v>Test Statistic</v>
+      </c>
+      <c r="C7" s="79"/>
+      <c r="D7" s="80"/>
+      <c r="E7" s="81"/>
+      <c r="F7" s="81"/>
+      <c r="G7" s="82"/>
+      <c r="H7" s="34" t="str" cm="1">
+        <f t="array" ref="H7:H10">TRIM(TRANSPOSE(D26:G26))</f>
+        <v>U = 260,162</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B8" s="78" t="str">
+        <v>p-value</v>
+      </c>
+      <c r="C8" s="79"/>
+      <c r="D8" s="80"/>
+      <c r="E8" s="81"/>
+      <c r="F8" s="81"/>
+      <c r="G8" s="82"/>
+      <c r="H8" s="34" t="str">
+        <v>0.078</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" hidden="1" outlineLevel="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="78" t="str">
+        <v>Effect Size</v>
+      </c>
+      <c r="C9" s="79"/>
+      <c r="D9" s="80"/>
+      <c r="E9" s="81"/>
+      <c r="F9" s="81"/>
+      <c r="G9" s="82"/>
+      <c r="H9" s="34" t="str">
+        <v>-</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" ht="15" collapsed="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B10" s="83" t="str">
+        <v>Interpretation</v>
+      </c>
+      <c r="C10" s="84"/>
+      <c r="D10" s="85"/>
+      <c r="E10" s="86"/>
+      <c r="F10" s="86"/>
+      <c r="G10" s="87"/>
+      <c r="H10" s="39" t="str">
+        <v>Marginally significant</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" s="55" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B16" s="55" t="s">
+        <v>863</v>
+      </c>
+      <c r="C16" s="67" t="s">
+        <v>874</v>
+      </c>
+      <c r="D16" s="68" t="s">
+        <v>875</v>
+      </c>
+      <c r="E16" s="55" t="s">
+        <v>876</v>
+      </c>
+      <c r="F16" s="55" t="s">
+        <v>877</v>
+      </c>
+      <c r="G16" s="55" t="s">
+        <v>878</v>
+      </c>
+      <c r="H16" s="68" t="s">
+        <v>879</v>
+      </c>
+      <c r="I16" s="68"/>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B17" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C17" s="57" t="s">
+        <v>795</v>
+      </c>
+      <c r="D17" s="40" t="s">
+        <v>775</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>775</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>807</v>
+      </c>
+      <c r="G17" s="20" t="s">
+        <v>795</v>
+      </c>
+      <c r="H17" s="40" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B18" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C18" s="57" t="s">
+        <v>880</v>
+      </c>
+      <c r="D18" s="40">
+        <v>154</v>
+      </c>
+      <c r="E18" s="20">
+        <v>860</v>
+      </c>
+      <c r="F18" s="20">
+        <v>5.4999999999999997E-3</v>
+      </c>
+      <c r="G18" s="20">
+        <v>2.3E-3</v>
+      </c>
+      <c r="H18" s="40">
+        <v>0.1134</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B19" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C19" s="57" t="s">
+        <v>881</v>
+      </c>
+      <c r="D19" s="40">
+        <v>112</v>
+      </c>
+      <c r="E19" s="20">
+        <v>639</v>
+      </c>
+      <c r="F19" s="20">
+        <v>1.52E-2</v>
+      </c>
+      <c r="G19" s="20">
+        <v>1.8499999999999999E-2</v>
+      </c>
+      <c r="H19" s="40">
+        <v>0.1111</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B20" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C20" s="57" t="s">
+        <v>882</v>
+      </c>
+      <c r="D20" s="40" t="s">
+        <v>883</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>883</v>
+      </c>
+      <c r="F20" s="20">
+        <v>-9.5999999999999992E-3</v>
+      </c>
+      <c r="G20" s="20">
+        <v>-1.6199999999999999E-2</v>
+      </c>
+      <c r="H20" s="40" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" s="55" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="B23" s="55" t="s">
+        <v>857</v>
+      </c>
+      <c r="C23" s="67" t="s">
+        <v>858</v>
+      </c>
+      <c r="D23" s="68" t="s">
+        <v>859</v>
+      </c>
+      <c r="E23" s="55" t="s">
+        <v>860</v>
+      </c>
+      <c r="F23" s="55" t="s">
+        <v>861</v>
+      </c>
+      <c r="G23" s="55" t="s">
+        <v>862</v>
+      </c>
+      <c r="H23" s="68"/>
+      <c r="I23" s="68"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B24" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C24" s="57" t="s">
+        <v>864</v>
+      </c>
+      <c r="D24" s="40" t="s">
+        <v>865</v>
+      </c>
+      <c r="E24" s="20" t="s">
+        <v>775</v>
+      </c>
+      <c r="F24" s="20" t="s">
+        <v>866</v>
+      </c>
+      <c r="G24" s="20" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B25" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C25" s="57" t="s">
+        <v>867</v>
+      </c>
+      <c r="D25" s="40" t="s">
+        <v>868</v>
+      </c>
+      <c r="E25" s="20">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="F25" s="20" t="s">
+        <v>869</v>
+      </c>
+      <c r="G25" s="20" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="B26" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C26" s="57" t="s">
+        <v>871</v>
+      </c>
+      <c r="D26" s="40" t="s">
+        <v>872</v>
+      </c>
+      <c r="E26" s="20">
+        <v>7.8E-2</v>
+      </c>
+      <c r="F26" s="20" t="s">
+        <v>873</v>
+      </c>
+      <c r="G26" s="20" t="s">
+        <v>885</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A65AF39-4FCA-4ECA-9A3F-8206E401F864}">
+  <dimension ref="B1:I10"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="20"/>
+    <col min="2" max="2" width="19.36328125" style="20" customWidth="1"/>
+    <col min="3" max="4" width="21.08984375" style="20" customWidth="1"/>
+    <col min="5" max="8" width="14.90625" style="20" customWidth="1"/>
+    <col min="9" max="16384" width="8.7265625" style="20"/>
+  </cols>
+  <sheetData>
     <row r="1" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C2" s="63" t="s">
-        <v>857</v>
-      </c>
-      <c r="D2" s="63"/>
-      <c r="E2" s="63"/>
-      <c r="F2" s="63"/>
-      <c r="G2" s="63"/>
-      <c r="H2" s="64"/>
-      <c r="I2"/>
-    </row>
-    <row r="3" spans="2:9" s="55" customFormat="1" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="65" t="s">
-        <v>845</v>
-      </c>
-      <c r="C3" s="61" t="str" cm="1">
-        <f t="array" ref="C3:H3">_xlfn.SEQUENCE(1,6,1970,10)&amp;"'s"</f>
-        <v>1970's</v>
-      </c>
-      <c r="D3" s="61" t="str">
-        <v>1980's</v>
-      </c>
-      <c r="E3" s="61" t="str">
-        <v>1990's</v>
-      </c>
-      <c r="F3" s="61" t="str">
-        <v>2000's</v>
-      </c>
-      <c r="G3" s="61" t="str">
-        <v>2010's</v>
-      </c>
-      <c r="H3" s="62" t="str">
-        <v>2020's</v>
-      </c>
-      <c r="I3" s="73" t="s">
-        <v>856</v>
-      </c>
-    </row>
-    <row r="4" spans="2:9" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="66" t="s">
-        <v>847</v>
-      </c>
-      <c r="C4" s="69" cm="1">
-        <f t="array" ref="C4:H6">C11:H13</f>
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="D4" s="69">
-        <v>0.46</v>
-      </c>
-      <c r="E4" s="69">
-        <v>0.19</v>
-      </c>
-      <c r="F4" s="69">
-        <v>0.08</v>
-      </c>
-      <c r="G4" s="69">
-        <v>0.53</v>
-      </c>
-      <c r="H4" s="45">
-        <v>0.16</v>
-      </c>
-      <c r="I4" s="72">
-        <f t="shared" ref="I4:I6" si="0">H4-C4</f>
-        <v>-0.40999999999999992</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B5" s="67" t="s">
-        <v>848</v>
-      </c>
-      <c r="C5" s="70">
-        <v>-0.35</v>
-      </c>
-      <c r="D5" s="70">
-        <v>0.42</v>
-      </c>
-      <c r="E5" s="70">
-        <v>-0.14000000000000001</v>
-      </c>
-      <c r="F5" s="70">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="G5" s="70">
-        <v>0.25</v>
-      </c>
-      <c r="H5" s="46">
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="I5" s="46">
-        <f t="shared" si="0"/>
-        <v>0.91999999999999993</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="68" t="s">
-        <v>849</v>
-      </c>
-      <c r="C6" s="71">
-        <v>0.02</v>
-      </c>
-      <c r="D6" s="71">
-        <v>-0.11</v>
-      </c>
-      <c r="E6" s="71">
-        <v>0.51</v>
-      </c>
-      <c r="F6" s="71">
-        <v>0.04</v>
-      </c>
-      <c r="G6" s="71">
-        <v>0.43</v>
-      </c>
-      <c r="H6" s="47">
-        <v>-7.0000000000000007E-2</v>
-      </c>
-      <c r="I6" s="47">
-        <f t="shared" si="0"/>
-        <v>-9.0000000000000011E-2</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:9" s="55" customFormat="1" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="51" t="str" cm="1">
+        <f t="array" ref="B2:H5">TRIM(C7:I10)</f>
+        <v>Validation Strategy</v>
+      </c>
+      <c r="C2" s="52" t="str">
+        <v>Training Samples</v>
+      </c>
+      <c r="D2" s="52" t="str">
+        <v>Test Samples</v>
+      </c>
+      <c r="E2" s="52" t="str">
+        <v>Train R²</v>
+      </c>
+      <c r="F2" s="52" t="str">
+        <v>Test R²</v>
+      </c>
+      <c r="G2" s="52" t="str">
+        <v>Test RMSE</v>
+      </c>
+      <c r="H2" s="54" t="str">
+        <v>Generalization Gap</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9" ht="28.5" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="108" t="str">
+        <v>Temporal Holdout (2020-2024)</v>
+      </c>
+      <c r="C3" s="105" t="str">
+        <v>1,523 seasons 
+(1970-2019)</v>
+      </c>
+      <c r="D3" s="105" t="str">
+        <v>160 seasons
+(2020-2024)</v>
+      </c>
+      <c r="E3" s="27" t="str">
+        <v>0.824</v>
+      </c>
+      <c r="F3" s="28" t="str">
+        <v>0.731</v>
+      </c>
+      <c r="G3" s="28" t="str">
+        <v>0.098</v>
+      </c>
+      <c r="H3" s="29" t="str">
+        <v>0.093</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" ht="28" x14ac:dyDescent="0.35">
+      <c r="B4" s="109" t="str">
+        <v>Holdout Coaches</v>
+      </c>
+      <c r="C4" s="106" t="str">
+        <v>1,363 seasons
+(216 coaches)</v>
+      </c>
+      <c r="D4" s="106" t="str">
+        <v>320 seasons
+(54 coaches)</v>
+      </c>
+      <c r="E4" s="32" t="str">
+        <v>0.816</v>
+      </c>
+      <c r="F4" s="33" t="str">
+        <v>0.745</v>
+      </c>
+      <c r="G4" s="33" t="str">
+        <v>0.097</v>
+      </c>
+      <c r="H4" s="34" t="str">
+        <v>0.071</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B5" s="110" t="str">
+        <v>New Coaches in Modern Era</v>
+      </c>
+      <c r="C5" s="107" t="str">
+        <v>1,652 seasons
+(pre-2020 + 80% of 2020-2024)</v>
+      </c>
+      <c r="D5" s="107" t="str">
+        <v>31 seasons
+(11 new coaches, 2020-2024)</v>
+      </c>
+      <c r="E5" s="37" t="str">
+        <v>0.811</v>
+      </c>
+      <c r="F5" s="38" t="str">
+        <v>0.771</v>
+      </c>
+      <c r="G5" s="38" t="str">
+        <v>0.093</v>
+      </c>
+      <c r="H5" s="39" t="str">
+        <v>0.041</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.35">
+      <c r="C7" s="20" t="s">
+        <v>937</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>938</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>939</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>940</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>941</v>
+      </c>
+      <c r="H7" s="20" t="s">
+        <v>942</v>
+      </c>
+      <c r="I7" s="20" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" ht="29" x14ac:dyDescent="0.35">
+      <c r="B8" s="20" t="s">
+        <v>863</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>944</v>
+      </c>
+      <c r="D8" s="55" t="s">
+        <v>947</v>
+      </c>
+      <c r="E8" s="55" t="s">
+        <v>950</v>
+      </c>
+      <c r="F8" s="20">
+        <v>0.82399999999999995</v>
+      </c>
+      <c r="G8" s="20">
+        <v>0.73099999999999998</v>
+      </c>
+      <c r="H8" s="20">
+        <v>9.8000000000000004E-2</v>
+      </c>
+      <c r="I8" s="20">
+        <v>9.2999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" ht="29" x14ac:dyDescent="0.35">
       <c r="B9" s="20" t="s">
-        <v>846</v>
-      </c>
-      <c r="C9" s="57" t="s">
-        <v>850</v>
-      </c>
-      <c r="D9" s="40" t="s">
-        <v>851</v>
-      </c>
-      <c r="E9" s="20" t="s">
-        <v>852</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>853</v>
-      </c>
-      <c r="G9" s="20" t="s">
-        <v>854</v>
-      </c>
-      <c r="H9" s="40" t="s">
-        <v>855</v>
-      </c>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.35">
+        <v>863</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>945</v>
+      </c>
+      <c r="D9" s="55" t="s">
+        <v>948</v>
+      </c>
+      <c r="E9" s="55" t="s">
+        <v>951</v>
+      </c>
+      <c r="F9" s="20">
+        <v>0.81599999999999995</v>
+      </c>
+      <c r="G9" s="20">
+        <v>0.745</v>
+      </c>
+      <c r="H9" s="20">
+        <v>9.7000000000000003E-2</v>
+      </c>
+      <c r="I9" s="20">
+        <v>7.0999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B10" s="20" t="s">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B11" s="20" t="s">
-        <v>847</v>
-      </c>
-      <c r="C11" s="57">
-        <v>0.56999999999999995</v>
-      </c>
-      <c r="D11" s="40">
-        <v>0.46</v>
-      </c>
-      <c r="E11" s="20">
-        <v>0.19</v>
-      </c>
-      <c r="F11" s="20">
-        <v>0.08</v>
-      </c>
-      <c r="G11" s="20">
-        <v>0.53</v>
-      </c>
-      <c r="H11" s="40">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B12" s="20" t="s">
-        <v>848</v>
-      </c>
-      <c r="C12" s="57">
-        <v>-0.35</v>
-      </c>
-      <c r="D12" s="40">
-        <v>0.42</v>
-      </c>
-      <c r="E12" s="20">
-        <v>-0.14000000000000001</v>
-      </c>
-      <c r="F12" s="20">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="G12" s="20">
-        <v>0.25</v>
-      </c>
-      <c r="H12" s="40">
-        <v>0.56999999999999995</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.35">
-      <c r="B13" s="20" t="s">
-        <v>849</v>
-      </c>
-      <c r="C13" s="57">
-        <v>0.02</v>
-      </c>
-      <c r="D13" s="40">
-        <v>-0.11</v>
-      </c>
-      <c r="E13" s="20">
-        <v>0.51</v>
-      </c>
-      <c r="F13" s="20">
-        <v>0.04</v>
-      </c>
-      <c r="G13" s="20">
-        <v>0.43</v>
-      </c>
-      <c r="H13" s="40">
-        <v>-7.0000000000000007E-2</v>
+        <v>863</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>946</v>
+      </c>
+      <c r="D10" s="55" t="s">
+        <v>949</v>
+      </c>
+      <c r="E10" s="55" t="s">
+        <v>952</v>
+      </c>
+      <c r="F10" s="20">
+        <v>0.81100000000000005</v>
+      </c>
+      <c r="G10" s="20">
+        <v>0.77100000000000002</v>
+      </c>
+      <c r="H10" s="20">
+        <v>9.2999999999999999E-2</v>
+      </c>
+      <c r="I10" s="20">
+        <v>4.1000000000000002E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>